<commit_message>
G3 core: scheduler with hard constraints, goal tree, finance maths (pure, property-tested)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -2624,7 +2624,7 @@
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Verified for G1 scope (automated evidence) — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="O25" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="O40" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Verified for G1 scope (automated evidence) — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -14726,10 +14726,14 @@
       <c r="H6" s="14" t="n"/>
       <c r="I6" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="n"/>
+          <t>Pass (G1) — G3 core: 100 generated plans, 0 tasks inside prayer/family/rest blocks, never over capacity, nothing silently dropped, deterministic</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>tests/g3.test.ts; src/core/planner.ts</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="n"/>
     </row>
     <row r="7" ht="21.75" customHeight="1" s="10">
@@ -15597,10 +15601,14 @@
       <c r="H25" s="14" t="n"/>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J25" s="14" t="n"/>
+          <t>Partial (G1) — Net-worth maths (personal/business separate, unknown→unknown) done; no screen yet</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>tests/g3.test.ts; src/core/finance.ts</t>
+        </is>
+      </c>
       <c r="K25" s="14" t="n"/>
     </row>
     <row r="26" ht="21.75" customHeight="1" s="10">
@@ -15642,10 +15650,14 @@
       <c r="H26" s="14" t="n"/>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J26" s="14" t="n"/>
+          <t>Partial (G1) — Monthly cash-flow + runway maths done; 90-day review screen not built</t>
+        </is>
+      </c>
+      <c r="J26" s="14" t="inlineStr">
+        <is>
+          <t>tests/g3.test.ts; src/core/finance.ts</t>
+        </is>
+      </c>
       <c r="K26" s="14" t="n"/>
     </row>
     <row r="27" ht="21.75" customHeight="1" s="10">
@@ -16276,10 +16288,14 @@
       <c r="H40" s="14" t="n"/>
       <c r="I40" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J40" s="14" t="n"/>
+          <t>Pass (G1) — G3 core: 200 random split/merge/delete ops, every task still reaches its goal, 0 orphans</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="inlineStr">
+        <is>
+          <t>tests/g3.test.ts; src/core/goals.ts</t>
+        </is>
+      </c>
       <c r="K40" s="14" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="10">

</xml_diff>

<commit_message>
Evidence: map TM-TST-171 to its tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -14420,7 +14420,7 @@
       </c>
       <c r="O174" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -22518,10 +22518,14 @@
       <c r="H174" s="14" t="n"/>
       <c r="I174" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J174" s="14" t="n"/>
+          <t>Partial (G1) — Home shows 1-3 own planned actions + current stage only (DOM test + browser e2e). 5-user 10-second usability test NOT run</t>
+        </is>
+      </c>
+      <c r="J174" s="14" t="inlineStr">
+        <is>
+          <t>tests/g1.test.ts; tests/g3ui.test.ts; tools/e2e.mjs</t>
+        </is>
+      </c>
       <c r="K174" s="14" t="n"/>
     </row>
     <row r="175" ht="21.75" customHeight="1" s="10">

</xml_diff>

<commit_message>
G3: Money screen (net worth, monthly cash flow; unknown stays unknown; personal/business apart)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -15601,12 +15601,12 @@
       <c r="H25" s="14" t="n"/>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>Partial (G1) — Net-worth maths (personal/business separate, unknown→unknown) done; no screen yet</t>
+          <t>Partial (G1) — Money screen: net worth per scope from saved items, unknown stays unknown, nothing-entered shows 'nothing yet'. Real-user test not run</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>tests/g3.test.ts; src/core/finance.ts</t>
+          <t>tests/g3.test.ts; tests/money.test.ts; tools/e2e.mjs</t>
         </is>
       </c>
       <c r="K25" s="14" t="n"/>
@@ -15650,12 +15650,12 @@
       <c r="H26" s="14" t="n"/>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>Partial (G1) — Monthly cash-flow + runway maths done; 90-day review screen not built</t>
+          <t>Partial (G1) — Monthly cash flow on screen (one-off/yearly counted aside). 90-day review view not built</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>tests/g3.test.ts; src/core/finance.ts</t>
+          <t>tests/g3.test.ts; tests/money.test.ts</t>
         </is>
       </c>
       <c r="K26" s="14" t="n"/>

</xml_diff>

<commit_message>
G3: stage rules (A auto-checked, B-H own evidence), journey log, Journey screen, Home reads real stage
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -14075,7 +14075,7 @@
       </c>
       <c r="O169" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -22293,10 +22293,14 @@
       <c r="H169" s="14" t="n"/>
       <c r="I169" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J169" s="14" t="n"/>
+          <t>Partial (G1) — Stage rules + journey log work: order fixed, evidence required, history append-only, calm copy (scan), before/after logged; browser e2e A-&gt;B. Stage templates beyond A are generic; usability test NOT run</t>
+        </is>
+      </c>
+      <c r="J169" s="14" t="inlineStr">
+        <is>
+          <t>tests/stages.test.ts; src/core/stages.ts; tools/e2e.mjs</t>
+        </is>
+      </c>
       <c r="K169" s="14" t="n"/>
     </row>
     <row r="170" ht="21.75" customHeight="1" s="10">

</xml_diff>

<commit_message>
Life Success system: integration plan, 21-category library skeleton, new requirements 173-180
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -2312,7 +2312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O175"/>
+  <dimension ref="A1:O183"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="9" min="1" max="1"/>
@@ -14492,6 +14492,430 @@
         </is>
       </c>
       <c r="O175" s="14" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>TM-REQ-173</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Life-Success knowledge library with one shared tag system (categories ≠ menu items)</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr"/>
+      <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>TM-REQ-174</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>'I'm stuck' problem loop: Identify → Diagnose → Intervene → Execute → Measure</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>TM-REQ-175</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Rule-based diagnosis of stuck causes; unknown answers never forced into a cause</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>TM-REQ-176</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Every library entry has evidence level, sources+date and safety notes; unverified never shown as advice</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>TM-REQ-177</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Emotional/health content shows professional-help notice and needs human review before shipping</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>TM-REQ-178</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Habits use recovery/restart plans; no streak counters or shaming copy</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr"/>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>TM-REQ-179</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Skill-gap and knowledge-gap maps with text equivalents</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr"/>
+      <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>TM-REQ-180</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>After missed days the app asks gently what got in the way (sleep, load, unclear step…)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr"/>
+      <c r="M183" t="inlineStr"/>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr">
         <is>
           <t>Not verified — no build</t>
         </is>

</xml_diff>

<commit_message>
Quick capture (free note → confirmed amounts/dates/decisions), Decisions & numbers report, field rules
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -2312,7 +2312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O183"/>
+  <dimension ref="A1:O185"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="9" min="1" max="1"/>
@@ -14916,6 +14916,112 @@
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr"/>
       <c r="O183" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>TM-REQ-181</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Quick capture: free note/decision → rule-based extraction of amounts, percents, durations, dates, decisions → user confirms → reports use only confirmed items; original note stays on device</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>TM-REQ-182</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Field rules: one fact per field, taps over typing, short text ≤80 chars, every field shows what/why/example/format</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr">
         <is>
           <t>Not verified — no build</t>
         </is>

</xml_diff>

<commit_message>
Scope the Life Success brief to what fits; add 'I'm stuck' (6 taps, rule-based, never adds work when tired)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -2312,7 +2312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O185"/>
+  <dimension ref="A1:O180"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="9" min="1" max="1"/>
@@ -14500,7 +14500,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>TM-REQ-173</t>
+          <t>TM-REQ-174</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -14510,7 +14510,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Life-Success knowledge library with one shared tag system (categories ≠ menu items)</t>
+          <t>'I'm stuck' problem loop: Identify → Diagnose → Intervene → Execute → Measure</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -14553,7 +14553,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>TM-REQ-174</t>
+          <t>TM-REQ-175</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -14563,7 +14563,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>'I'm stuck' problem loop: Identify → Diagnose → Intervene → Execute → Measure</t>
+          <t>Rule-based diagnosis of stuck causes; unknown answers never forced into a cause</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -14606,7 +14606,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>TM-REQ-175</t>
+          <t>TM-REQ-178</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -14616,7 +14616,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Rule-based diagnosis of stuck causes; unknown answers never forced into a cause</t>
+          <t>Habits use recovery/restart plans; no streak counters or shaming copy</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -14659,7 +14659,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>TM-REQ-176</t>
+          <t>TM-REQ-181</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -14669,7 +14669,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Every library entry has evidence level, sources+date and safety notes; unverified never shown as advice</t>
+          <t>Quick capture: free note/decision → rule-based extraction of amounts, percents, durations, dates, decisions → user confirms → reports use only confirmed items; original note stays on device</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -14712,7 +14712,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>TM-REQ-177</t>
+          <t>TM-REQ-182</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -14722,7 +14722,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Emotional/health content shows professional-help notice and needs human review before shipping</t>
+          <t>Field rules: one fact per field, taps over typing, short text ≤80 chars, every field shows what/why/example/format</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -14738,12 +14738,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -14757,271 +14757,6 @@
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr">
-        <is>
-          <t>Not verified — no build</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>TM-REQ-178</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>Life Success system</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>Habits use recovery/restart plans; no streak counters or shaming copy</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>FIRST-BUILD (G1-G3)</t>
-        </is>
-      </c>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
-      <c r="M181" t="inlineStr"/>
-      <c r="N181" t="inlineStr"/>
-      <c r="O181" t="inlineStr">
-        <is>
-          <t>Not verified — no build</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>TM-REQ-179</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>Life Success system</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>Skill-gap and knowledge-gap maps with text equivalents</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="G182" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>FIRST-BUILD (G1-G3)</t>
-        </is>
-      </c>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr"/>
-      <c r="M182" t="inlineStr"/>
-      <c r="N182" t="inlineStr"/>
-      <c r="O182" t="inlineStr">
-        <is>
-          <t>Not verified — no build</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>TM-REQ-180</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>Life Success system</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>After missed days the app asks gently what got in the way (sleep, load, unclear step…)</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr"/>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>FIRST-BUILD (G1-G3)</t>
-        </is>
-      </c>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
-      <c r="M183" t="inlineStr"/>
-      <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr">
-        <is>
-          <t>Not verified — no build</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>TM-REQ-181</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>Life Success system</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>Quick capture: free note/decision → rule-based extraction of amounts, percents, durations, dates, decisions → user confirms → reports use only confirmed items; original note stays on device</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>FIRST-BUILD (G1-G3)</t>
-        </is>
-      </c>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
-      <c r="M184" t="inlineStr"/>
-      <c r="N184" t="inlineStr"/>
-      <c r="O184" t="inlineStr">
-        <is>
-          <t>Not verified — no build</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>TM-REQ-182</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>Life Success system</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Field rules: one fact per field, taps over typing, short text ≤80 chars, every field shows what/why/example/format</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>FIRST-BUILD (G1-G3)</t>
-        </is>
-      </c>
-      <c r="J185" t="inlineStr"/>
-      <c r="K185" t="inlineStr"/>
-      <c r="L185" t="inlineStr"/>
-      <c r="M185" t="inlineStr"/>
-      <c r="N185" t="inlineStr"/>
-      <c r="O185" t="inlineStr">
         <is>
           <t>Not verified — no build</t>
         </is>

</xml_diff>

<commit_message>
Topics library (21 topics, tips+visuals, tags), hideable drawer, task Done + reward picture (stars + garden layers)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_G1_evidence.xlsx
@@ -2312,7 +2312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O180"/>
+  <dimension ref="A1:O183"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="9" min="1" max="1"/>
@@ -14757,6 +14757,165 @@
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>TM-REQ-183</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Topic library: every owner topic (20 + Deen) has short practical tips with a visual; tips share tags so related tips appear across topics; all drafts marked unreviewed; sensitive topics carry safety notes</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr"/>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>TM-REQ-184</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Reward picture: each finished task adds a star, each passed stage adds a garden layer; milestone moments; no points/ranks/streaks/comparison; text equivalent</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr"/>
+      <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Not verified — no build</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>TM-REQ-185</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Life Success system</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Hideable side drawer listing all topics while the 5 phone tabs stay primary</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>FIRST-BUILD (G1-G3)</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr"/>
+      <c r="M183" t="inlineStr"/>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr">
         <is>
           <t>Not verified — no build</t>
         </is>

</xml_diff>